<commit_message>
Update best_opportinities.xlsx with new data revisions
- Modified the `best_opportinities.xlsx` file to include the latest updates on funding opportunities, ensuring the data remains accurate and user-friendly.
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -1,11 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D82A18-853C-448A-81DC-0C9DC4EDCBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Opportunities" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Scan Notes" state="visible" r:id="rId5"/>
+    <sheet name="Opportunities" sheetId="1" r:id="rId1"/>
+    <sheet name="Scan Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -242,19 +246,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -268,14 +272,26 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -340,10 +356,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -379,8 +396,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -717,19 +738,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="42.142857142857146" customWidth="1"/>
+    <col min="1" max="3" width="42.1796875" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="10" max="24" width="13.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -758,7 +779,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -787,11 +808,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="157" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -812,7 +833,7 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>24</v>
       </c>
@@ -837,7 +858,7 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>28</v>
       </c>
@@ -862,7 +883,7 @@
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
     </row>
-    <row r="6" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>32</v>
       </c>
@@ -889,7 +910,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
@@ -914,7 +935,7 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" ht="92.25" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
@@ -939,41 +960,44 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="92.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="11" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="13" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="14" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="15" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="18" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="19" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="20" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="21" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="22" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="23" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="25" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <autoFilter ref="A1:I8"/>
+  <autoFilter ref="A1:I8" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{69122B11-ADD0-416B-9282-2A1D1AE19D68}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="42.142857142857146" customWidth="1"/>
-    <col min="3" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="2" max="2" width="42.1796875" customWidth="1"/>
+    <col min="3" max="24" width="13.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>45</v>
       </c>
@@ -981,7 +1005,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>47</v>
       </c>
@@ -989,7 +1013,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>49</v>
       </c>
@@ -997,7 +1021,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>51</v>
       </c>
@@ -1005,7 +1029,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>53</v>
       </c>
@@ -1013,7 +1037,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>55</v>
       </c>
@@ -1021,7 +1045,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>57</v>
       </c>
@@ -1029,7 +1053,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>59</v>
       </c>
@@ -1037,7 +1061,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>61</v>
       </c>
@@ -1045,7 +1069,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>63</v>
       </c>
@@ -1053,7 +1077,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>65</v>
       </c>
@@ -1061,7 +1085,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>67</v>
       </c>
@@ -1069,7 +1093,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>69</v>
       </c>
@@ -1077,7 +1101,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>71</v>
       </c>
@@ -1085,7 +1109,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
         <v>73</v>
       </c>
@@ -1095,6 +1119,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update best_opportunities.xlsx with new data entries
- Revised the `best_opportunities.xlsx` file to include updated information on funding opportunities, enhancing the resource for FairBanks' initiatives.
- Ensured the new entries align with current project goals and community engagement strategies.
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D82A18-853C-448A-81DC-0C9DC4EDCBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0385450F-CFF5-4E2D-8310-D94F15F685EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -360,7 +360,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -397,6 +397,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -837,7 +843,7 @@
       <c r="A4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="13" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -862,7 +868,7 @@
       <c r="A5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="14" t="s">
         <v>29</v>
       </c>
       <c r="C5" s="6" t="s">
@@ -887,7 +893,7 @@
       <c r="A6" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="15" t="s">
         <v>33</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -914,7 +920,7 @@
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="13" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -939,7 +945,7 @@
       <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="13" t="s">
         <v>42</v>
       </c>
       <c r="C8" s="4" t="s">
@@ -981,6 +987,11 @@
   <autoFilter ref="A1:I8" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{69122B11-ADD0-416B-9282-2A1D1AE19D68}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{9ACED294-212B-4719-8A88-1FD72E17257B}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{F8D817B4-147D-4E4D-B65D-6D3D264C9FBB}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{849D98B6-B164-4F9F-ACC1-23668E839F27}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{A75DAD3F-EB59-4423-A0CF-CBF61E5B0CB6}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{5B1F9988-0430-4CE2-A0DB-D32777B5B670}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
Update evaluation documents and best opportunities file
- Revised `best_opportinities.xlsx` to reflect new data entries, enhancing resource availability for FairBanks' initiatives.
- Improved layout and content in `internal_staff_evaluation_fillable.pdf`, including updated contact information and formatting adjustments for better usability and clarity.
- Ensured all changes align with FairBanks' commitment to effective feedback collection and community engagement.
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0385450F-CFF5-4E2D-8310-D94F15F685EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD4251E-3350-48E9-964F-A5DE0979A275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -864,7 +864,7 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="155" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>28</v>
       </c>
@@ -889,7 +889,7 @@
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
     </row>
-    <row r="6" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="169.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>32</v>
       </c>
@@ -916,7 +916,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="156.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>

</xml_diff>

<commit_message>
Update pitch deck and documentation for FCHIP project
- Revised `build_africa-health-tech-accelerator_docs.py` to enhance the clarity of outcomes and strengths, replacing outdated text with updated messaging focused on evidence for buyers and partners.
- Updated the `FairBanks_FCHIP_Africa_Health_Tech_Accelerator_2026_Pitch.pdf` to reflect these changes, ensuring alignment with the project's goals and readiness for Demo Day.
- Modified the `best_opportinities.xlsx` to include new data entries, improving resource availability for funding opportunities.
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD4251E-3350-48E9-964F-A5DE0979A275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9489B389-7F40-4058-8025-0C8CD5247DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="77">
   <si>
     <t>Project Title</t>
   </si>
@@ -66,9 +66,6 @@
     <t>Submitted</t>
   </si>
   <si>
-    <t>13/July/2027</t>
-  </si>
-  <si>
     <t>applications/awief</t>
   </si>
   <si>
@@ -241,6 +238,15 @@
   </si>
   <si>
     <t>Rebuild via opportunities/build_opportunities.py (canonical). Peri-urban companion file removed after merge.</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>applications/africa-health-tech-accelerator/pitch-deck</t>
+  </si>
+  <si>
+    <t>MVP - pitch deck</t>
   </si>
 </sst>
 </file>
@@ -360,7 +366,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -403,6 +409,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -789,7 +804,7 @@
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="16" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -802,166 +817,170 @@
         <v>13</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="18">
+        <v>46216</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="157" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>22</v>
+        <v>76</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+        <v>15</v>
+      </c>
+      <c r="H3" s="17">
+        <v>46223</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="4" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="E4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
     <row r="5" spans="1:9" ht="155" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
     </row>
     <row r="6" spans="1:9" ht="169.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="C6" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>35</v>
-      </c>
       <c r="E6" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>14</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="156.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="C7" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="E7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>44</v>
-      </c>
       <c r="E8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -992,6 +1011,7 @@
     <hyperlink ref="B6" r:id="rId4" xr:uid="{849D98B6-B164-4F9F-ACC1-23668E839F27}"/>
     <hyperlink ref="B7" r:id="rId5" xr:uid="{A75DAD3F-EB59-4423-A0CF-CBF61E5B0CB6}"/>
     <hyperlink ref="B8" r:id="rId6" xr:uid="{5B1F9988-0430-4CE2-A0DB-D32777B5B670}"/>
+    <hyperlink ref="B2" r:id="rId7" xr:uid="{96CF7E40-08DF-4809-BE5E-9C241326465F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -1010,122 +1030,122 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>49</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>53</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>55</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>57</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>59</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>61</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>63</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>65</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>67</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>69</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>71</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>73</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add application letter, CV, and course units for Wasswa Wilson
- Created a new application letter for the Field Sales Supervisor position at Omel Medical Equipment Limited.
- Added a comprehensive CV detailing educational background, work experience, and skills relevant to biomedical engineering and software development.
- Included a document listing course units completed during the Biomedical Engineering program to showcase academic qualifications.
- Introduced additional identification and supporting documents to enhance the application package.
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9489B389-7F40-4058-8025-0C8CD5247DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BE2757-BDC8-42F9-A16E-C99EEA044D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="78">
   <si>
     <t>Project Title</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>MVP - pitch deck</t>
+  </si>
+  <si>
+    <t>Submitted PoC</t>
   </si>
 </sst>
 </file>
@@ -875,12 +878,14 @@
         <v>20</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="4"/>
+        <v>15</v>
+      </c>
+      <c r="H4" s="17">
+        <v>46223</v>
+      </c>
       <c r="I4" s="4"/>
     </row>
     <row r="5" spans="1:9" ht="155" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update best_opportunities.xlsx with new data and insights for partnership evaluation
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -20,9 +20,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,12 @@
       <u val="single"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -107,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -130,12 +136,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -193,6 +213,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -598,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="42.1796875" customWidth="1" min="1" max="3"/>
@@ -986,8 +1021,96 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="92.25" customHeight="1"/>
-    <row r="11" ht="92.25" customHeight="1"/>
+    <row r="10" ht="110" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Jay Shetty / GS Media — Strategic Partnership Outreach</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>https://www.jayshetty.me/</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Strategic partnership outreach to Jay Shetty and GS Media on community wellbeing, preventive healthcare, storytelling, and social-impact collaboration. FairBanks brings a live medical centre, Community Reach (CHWs/VHTs, outreach, CHIS, livelihoods), and an FCHIP MVP in development. This is a rolling partnership pitch, not a timed grant call. Prepared pack under applications/jayshetty; outreach email submitted with the PDF brief.</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Rolling (partnership outreach)</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G10" s="21" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>46225</v>
+      </c>
+      <c r="I10" s="21" t="inlineStr">
+        <is>
+          <t>applications/jayshetty</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="110" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Yunus Centre — Social Business Partnership Outreach</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>https://www.muhammadyunus.org/</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>Partnership exploration with Yunus Centre, the global hub for social business, on community health as a social business in Uganda. Focus areas: CHIS and livelihoods, learning exchange, YSBC/network introductions, and advice while developing the FCHIP MVP. Rolling outreach via official Yunus Centre channels (info@yunuscentre.org). Prepared pack under applications/yunus; outreach email submitted with the PDF brief.</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Rolling (partnership outreach)</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="n">
+        <v>46225</v>
+      </c>
+      <c r="I11" s="21" t="inlineStr">
+        <is>
+          <t>applications/yunus</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="92.25" customHeight="1"/>
     <row r="13" ht="92.25" customHeight="1"/>
     <row r="14" ht="92.25" customHeight="1"/>
@@ -1024,7 +1147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1052,7 +1175,7 @@
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>2026-07-19 21:46</t>
+          <t>2026-07-22 (added Jay Shetty + Yunus Centre submissions)</t>
         </is>
       </c>
     </row>
@@ -1209,6 +1332,18 @@
       <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Rebuild via opportunities/build_opportunities.py (canonical). Peri-urban companion file removed after merge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>Recent partnership submissions</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-22: Submitted Jay Shetty strategic partnership pack (applications/jayshetty) and Yunus Centre social business partnership pack (applications/yunus). Both marked Complete / Submitted in Opportunities.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update best_opportunities.xlsx with the latest data revisions.
</commit_message>
<xml_diff>
--- a/opportunities/best_opportinities.xlsx
+++ b/opportunities/best_opportinities.xlsx
@@ -155,7 +155,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -228,6 +228,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -633,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="42.1796875" customWidth="1" min="1" max="3"/>
@@ -862,224 +865,224 @@
       <c r="I5" s="6" t="n"/>
     </row>
     <row r="6" ht="169.5" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DPI Safeguards Accelerator (UN ODET / UNDP)</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>https://www.dpi-safeguards.org/accelerator</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Cohort programme helping partners embed practical safeguards into active Digital Public Infrastructure. NGO pathway for Uganda: issue-specific work on FairBanks FCHIP (consent/data use, offline inclusion, grievance). Catalytic grant up to USD 70,000 over 6-9 months, plus tools and peer learning. Stage 1 Airtable screening; Stage 2 needs government letter if longlisted. FairBanks submitted as community-based health operator with live FCHIP MVP.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>30 July 2026</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>applications/dpi-safeguards</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="156.5" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>U.S. Dept of State — Uganda Health System MOU (up to $60M)</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>https://opportunitiesforyouth.org/2026/06/15/u-s-department-of-state-launches-up-to-60-million-funding-opportunity-to-strengthen-ugandas-health-system-through-the-health-foreign-assistance-mou-implementation-plan/</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Major U.S. Department of State call (DFOP0017890) to strengthen Uganda's health system under the U.S.–Uganda Health MOU: up to $60M across ~15 awards over five years. Objective 4 funds scaling digital health systems (EMRs, DHIS2, eCHIS, iHRIS, national data warehouse); other tracks cover community-based health financing, faith/community facilities, and supply-chain accountability. Two-step process starting with a Statement of Interest. Highly aligned with FCHIP and FairBanks community health work. Ugandan organisations are the intended applicants.</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>31 July 2026 (Statement of Interest, 5:00 PM EDT)</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Drafting</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>applications/dos-uganda</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="156.5" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Embassy of Japan in Uganda — Grant Assistance for Grass-roots Human Security Projects (GGP)</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>https://www.ug.emb-japan.go.jp/itpr_en/ggp_en.html</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Japanese Embassy grant for non-profit, development-oriented organisations running community projects in Uganda that directly help people at the grassroots. Priority areas typically include basic health, education, water/sanitation, and related community infrastructure. Grants are usually up to about JPY 10 million per project, with selection twice a year. FairBanks Community Reach / facility-linked community health projects can fit if framed as grassroots benefit (not only software). Applications accepted year-round by email; selection after 15 Feb and 15 Jun deadlines.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>15 February / 15 June (rolling intake; next cycle 15 Feb 2027)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Multi-gender (all genders)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-      <c r="H7" s="20" t="n">
-        <v>46225</v>
-      </c>
-      <c r="I7" s="4" t="n"/>
     </row>
     <row r="8" ht="92.25" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>Embassy of Japan in Uganda — Grant Assistance for Grass-roots Human Security Projects (GGP)</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>https://www.ug.emb-japan.go.jp/itpr_en/ggp_en.html</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Japanese Embassy grant for non-profit, development-oriented organisations running community projects in Uganda that directly help people at the grassroots. Priority areas typically include basic health, education, water/sanitation, and related community infrastructure. Grants are usually up to about JPY 10 million per project, with selection twice a year. FairBanks Community Reach / facility-linked community health projects can fit if framed as grassroots benefit (not only software). Applications accepted year-round by email; selection after 15 Feb and 15 Jun deadlines.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>15 February / 15 June (rolling intake; next cycle 15 Feb 2027)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>46225</v>
+      </c>
+      <c r="I8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="92.25" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>Draper Richards Kaplan Foundation — Early-Stage Social Enterprises</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>https://www.drkfoundation.org/apply/</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Rolling philanthropic support (often cited up to about US$300,000) for early-stage social impact organisations solving urgent global problems with scalable models. Relevant if FairBanks/FCHIP presents as a social enterprise with a clear theory of change for community health intelligence in underserved peri-urban African settings. Highly selective; confirm current criteria and apply process on the official DRK Foundation website before preparing a full package.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Rolling</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="92.25" customHeight="1">
-      <c r="A9" t="inlineStr">
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="110" customHeight="1">
+      <c r="A10" t="inlineStr">
         <is>
           <t>DIV Fund (Development Innovation Ventures) — Open Innovation Grants</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>https://www.div.fund/apply</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Evidence-driven open innovation fund accepting applications year-round. Stages roughly: Pilot up to ~US$200,000; Testing higher; Scale up to about US$1.5 million. Funds innovations that can cost-effectively improve millions of lives in low- and middle-income countries. Open to nonprofits, startups, universities, and social enterprises — Ugandan applicants eligible. Good medium-term pathway for FCHIP if you can show a clear pilot plan, cost-effectiveness case, and path to scale across peri-urban and district health systems.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Rolling (applications accepted year-round)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Multi-gender (all genders)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="110" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>Jay Shetty / GS Media — Strategic Partnership Outreach</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="inlineStr">
-        <is>
-          <t>https://www.jayshetty.me/</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="inlineStr">
-        <is>
-          <t>Strategic partnership outreach to Jay Shetty and GS Media on community wellbeing, preventive healthcare, storytelling, and social-impact collaboration. FairBanks brings a live medical centre, Community Reach (CHWs/VHTs, outreach, CHIS, livelihoods), and an FCHIP MVP in development. This is a rolling partnership pitch, not a timed grant call. Prepared pack under applications/jayshetty; outreach email submitted with the PDF brief.</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="inlineStr">
-        <is>
-          <t>Rolling (partnership outreach)</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>Multi-gender (all genders)</t>
-        </is>
-      </c>
-      <c r="F10" s="21" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G10" s="21" t="inlineStr">
-        <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="n">
-        <v>46225</v>
-      </c>
-      <c r="I10" s="21" t="inlineStr">
-        <is>
-          <t>applications/jayshetty</t>
         </is>
       </c>
     </row>
     <row r="11" ht="110" customHeight="1">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>Yunus Centre — Social Business Partnership Outreach</t>
+          <t>Jay Shetty / GS Media — Strategic Partnership Outreach</t>
         </is>
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>https://www.muhammadyunus.org/</t>
+          <t>https://www.jayshetty.me/</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>Partnership exploration with Yunus Centre, the global hub for social business, on community health as a social business in Uganda. Focus areas: CHIS and livelihoods, learning exchange, YSBC/network introductions, and advice while developing the FCHIP MVP. Rolling outreach via official Yunus Centre channels (info@yunuscentre.org). Prepared pack under applications/yunus; outreach email submitted with the PDF brief.</t>
+          <t>Strategic partnership outreach to Jay Shetty and GS Media on community wellbeing, preventive healthcare, storytelling, and social-impact collaboration. FairBanks brings a live medical centre, Community Reach (CHWs/VHTs, outreach, CHIS, livelihoods), and an FCHIP MVP in development. This is a rolling partnership pitch, not a timed grant call. Prepared pack under applications/jayshetty; outreach email submitted with the PDF brief.</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
@@ -1107,11 +1110,55 @@
       </c>
       <c r="I11" s="21" t="inlineStr">
         <is>
+          <t>applications/jayshetty</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="92.25" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Yunus Centre — Social Business Partnership Outreach</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>https://www.muhammadyunus.org/</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>Partnership exploration with Yunus Centre, the global hub for social business, on community health as a social business in Uganda. Focus areas: CHIS and livelihoods, learning exchange, YSBC/network introductions, and advice while developing the FCHIP MVP. Rolling outreach via official Yunus Centre channels (info@yunuscentre.org). Prepared pack under applications/yunus; outreach email submitted with the PDF brief.</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Rolling (partnership outreach)</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>46225</v>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
+        <is>
           <t>applications/yunus</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="92.25" customHeight="1"/>
     <row r="13" ht="92.25" customHeight="1"/>
     <row r="14" ht="92.25" customHeight="1"/>
     <row r="15" ht="92.25" customHeight="1"/>
@@ -1147,7 +1194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1347,6 +1394,18 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DPI Safeguards Accelerator</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Added 2026-07-29 as Submitted (Stage 1 NGO pathway Airtable). Pack: applications/dpi-safeguards. Official: https://www.dpi-safeguards.org/accelerator. Ask USD 60k-70k / 7-9 months; issue-specific FCHIP safeguards; KCCA Central Division engagement initiating.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>